<commit_message>
Working to get multiple consequences on separate rows at Powell elevation 3490
</commit_message>
<xml_diff>
--- a/R-Figs/AutoReadUSBRData/ReservoirElevationDefinitions.xlsx
+++ b/R-Figs/AutoReadUSBRData/ReservoirElevationDefinitions.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Rosenberg\Work\USU\Research\ColoradoRiver\RCode\ColoradoRiverCollaborate\AutoReadUSBRData\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://api.box.com/wopi/files/2558006682865/WOPIServiceId_TP_BOX_2/WOPIUserId_-/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{93E988A9-6564-4F69-98E8-ABFBF40E39BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="3" documentId="13_ncr:1_{93E988A9-6564-4F69-98E8-ABFBF40E39BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{822D0CD4-E939-41F2-9472-2433B2782B4F}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-1965" windowWidth="29040" windowHeight="17520" activeTab="1" xr2:uid="{8459C475-5003-475B-AAB9-94E9EA45958F}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="2" xr2:uid="{8459C475-5003-475B-AAB9-94E9EA45958F}"/>
   </bookViews>
   <sheets>
     <sheet name="ReadMe" sheetId="2" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="36">
   <si>
     <t>Reservoir</t>
   </si>
@@ -108,12 +108,6 @@
     <t>No Hydropower (Vortices)</t>
   </si>
   <si>
-    <t>No hydropower generation or delivery to 9 western U.S. states</t>
-  </si>
-  <si>
-    <t>Vortices in penstocks</t>
-  </si>
-  <si>
     <t>Risk</t>
   </si>
   <si>
@@ -133,6 +127,9 @@
   </si>
   <si>
     <t>Invasive fish move into Grand Canyon and threaten native fish</t>
+  </si>
+  <si>
+    <t>No hydropower generation or transmission to 9 western U.S. states\\nInfrastructure operates outside design specs\\nReduced downstream delivery</t>
   </si>
 </sst>
 </file>
@@ -1053,7 +1050,7 @@
         <v>23</v>
       </c>
       <c r="D1" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.35">
@@ -1067,7 +1064,7 @@
         <v>895</v>
       </c>
       <c r="D2" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
@@ -1081,7 +1078,7 @@
         <v>950</v>
       </c>
       <c r="D3" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">
@@ -1161,7 +1158,7 @@
         <v>1135</v>
       </c>
       <c r="D10" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.35">
@@ -1217,7 +1214,7 @@
         <v>23</v>
       </c>
       <c r="D1" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.35">
@@ -1231,7 +1228,7 @@
         <v>3370</v>
       </c>
       <c r="D2" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
@@ -1245,7 +1242,7 @@
         <v>3490</v>
       </c>
       <c r="D3" t="s">
-        <v>28</v>
+        <v>35</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">
@@ -1269,9 +1266,6 @@
       <c r="C5">
         <v>3514</v>
       </c>
-      <c r="D5" t="s">
-        <v>29</v>
-      </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
@@ -1284,7 +1278,7 @@
         <v>3525</v>
       </c>
       <c r="D6" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
Break consequences by line; working to add last day to monthly reservoir data frame
</commit_message>
<xml_diff>
--- a/R-Figs/AutoReadUSBRData/ReservoirElevationDefinitions.xlsx
+++ b/R-Figs/AutoReadUSBRData/ReservoirElevationDefinitions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://api.box.com/wopi/files/2558006682865/WOPIServiceId_TP_BOX_2/WOPIUserId_-/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3" documentId="13_ncr:1_{93E988A9-6564-4F69-98E8-ABFBF40E39BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{822D0CD4-E939-41F2-9472-2433B2782B4F}"/>
+  <xr:revisionPtr revIDLastSave="4" documentId="13_ncr:1_{93E988A9-6564-4F69-98E8-ABFBF40E39BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6885C9C5-7B1B-4BEF-83B7-55829272D81E}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="2" xr2:uid="{8459C475-5003-475B-AAB9-94E9EA45958F}"/>
   </bookViews>
@@ -129,7 +129,7 @@
     <t>Invasive fish move into Grand Canyon and threaten native fish</t>
   </si>
   <si>
-    <t>No hydropower generation or transmission to 9 western U.S. states\\nInfrastructure operates outside design specs\\nReduced downstream delivery</t>
+    <t>No hydropower generation or transmission to 9 western U.S. states;Infrastructure operates outside design specs;Reduced downstream delivery</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
Lake Powell consequence figure showing well in R file
</commit_message>
<xml_diff>
--- a/R-Figs/AutoReadUSBRData/ReservoirElevationDefinitions.xlsx
+++ b/R-Figs/AutoReadUSBRData/ReservoirElevationDefinitions.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://api.box.com/wopi/files/2558006682865/WOPIServiceId_TP_BOX_2/WOPIUserId_-/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="4" documentId="13_ncr:1_{93E988A9-6564-4F69-98E8-ABFBF40E39BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6885C9C5-7B1B-4BEF-83B7-55829272D81E}"/>
+  <xr:revisionPtr revIDLastSave="12" documentId="13_ncr:1_{93E988A9-6564-4F69-98E8-ABFBF40E39BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BCE918C2-1536-4AC5-8DC7-36E43C63DC0B}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="2" xr2:uid="{8459C475-5003-475B-AAB9-94E9EA45958F}"/>
+    <workbookView xWindow="-57720" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{8459C475-5003-475B-AAB9-94E9EA45958F}"/>
   </bookViews>
   <sheets>
     <sheet name="ReadMe" sheetId="2" r:id="rId1"/>
@@ -111,25 +111,25 @@
     <t>Risk</t>
   </si>
   <si>
-    <t>No downstream delivery to Lower Basin states and Mexico</t>
-  </si>
-  <si>
     <t>No downstream delivery to CA, AZ, NV, and Mexico</t>
   </si>
   <si>
     <t>No hydropower generation and delivery to Los Angeles, Las Vegas, or Phoenix</t>
   </si>
   <si>
-    <t>Invasive fish pass though dam, spread, and threaten native fish</t>
-  </si>
-  <si>
     <t>Consequence</t>
   </si>
   <si>
     <t>Invasive fish move into Grand Canyon and threaten native fish</t>
   </si>
   <si>
-    <t>No hydropower generation or transmission to 9 western U.S. states;Infrastructure operates outside design specs;Reduced downstream delivery</t>
+    <t>No downstream delivery to Lower Basin states and Mexico.</t>
+  </si>
+  <si>
+    <t>No hydropower generation or transmission to 9 western U.S. states.;Infrastructure operates outside design criteria.;Reduced downstream delivery to Lower Basin states and Mexico.</t>
+  </si>
+  <si>
+    <t>Higher release temperatures.;Increased risk that invasive fish pass though dam, spawn,;spread, and threaten native fish</t>
   </si>
 </sst>
 </file>
@@ -1064,7 +1064,7 @@
         <v>895</v>
       </c>
       <c r="D2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
@@ -1078,7 +1078,7 @@
         <v>950</v>
       </c>
       <c r="D3" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">
@@ -1158,7 +1158,7 @@
         <v>1135</v>
       </c>
       <c r="D10" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.35">
@@ -1214,7 +1214,7 @@
         <v>23</v>
       </c>
       <c r="D1" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.35">
@@ -1228,7 +1228,7 @@
         <v>3370</v>
       </c>
       <c r="D2" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
@@ -1242,7 +1242,7 @@
         <v>3490</v>
       </c>
       <c r="D3" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">
@@ -1278,7 +1278,7 @@
         <v>3525</v>
       </c>
       <c r="D6" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
Figure 1 Powell over time in Rmd mostly working
</commit_message>
<xml_diff>
--- a/R-Figs/AutoReadUSBRData/ReservoirElevationDefinitions.xlsx
+++ b/R-Figs/AutoReadUSBRData/ReservoirElevationDefinitions.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://api.box.com/wopi/files/2558006682865/WOPIServiceId_TP_BOX_2/WOPIUserId_-/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="32" documentId="13_ncr:1_{93E988A9-6564-4F69-98E8-ABFBF40E39BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E5CC4C16-8AFD-4CE7-999C-08EA841C1D93}"/>
+  <xr:revisionPtr revIDLastSave="35" documentId="13_ncr:1_{93E988A9-6564-4F69-98E8-ABFBF40E39BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D577B65D-7E7C-41A5-A032-C630C2BCCC4D}"/>
   <bookViews>
-    <workbookView xWindow="-57720" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{8459C475-5003-475B-AAB9-94E9EA45958F}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{8459C475-5003-475B-AAB9-94E9EA45958F}"/>
   </bookViews>
   <sheets>
     <sheet name="ReadMe" sheetId="2" r:id="rId1"/>
@@ -118,15 +118,6 @@
     <t>Consequence</t>
   </si>
   <si>
-    <t>No downstream delivery to Lower Basin states and Mexico.</t>
-  </si>
-  <si>
-    <t>No hydropower generation or transmission to 9 western U.S. states.;Infrastructure operates outside design criteria.;Reduced downstream delivery to Lower Basin states and Mexico.</t>
-  </si>
-  <si>
-    <t>Higher release temperatures.;Increased risk that invasive fish pass though dam, spawn,;spread, and threaten native fish</t>
-  </si>
-  <si>
     <t>No downstream delivery to CA, AZ, and Mexico</t>
   </si>
   <si>
@@ -140,6 +131,15 @@
   </si>
   <si>
     <t>Invasive fish stop moving upstream into Grand Canyon;Potect native fish</t>
+  </si>
+  <si>
+    <t>No downstream delivery to;Lower Basin states and Mexico.</t>
+  </si>
+  <si>
+    <t>No hydropower generation or transmission; to 9 western U.S. states.;Infrastructure operates outside;design criteria.;Reduced downstream delivery to;Lower Basin states and Mexico.</t>
+  </si>
+  <si>
+    <t>Higher release temperatures.;Increased risk that invasive fish pass;though dam, spawn, spread, and;threaten native fish</t>
   </si>
 </sst>
 </file>
@@ -1074,7 +1074,7 @@
         <v>895</v>
       </c>
       <c r="D2" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
@@ -1088,7 +1088,7 @@
         <v>950</v>
       </c>
       <c r="D3" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">
@@ -1107,7 +1107,7 @@
         <v>1</v>
       </c>
       <c r="B5" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="C5">
         <v>1000</v>
@@ -1179,7 +1179,7 @@
         <v>1135</v>
       </c>
       <c r="D11" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.35">
@@ -1249,7 +1249,7 @@
         <v>3370</v>
       </c>
       <c r="D2" t="s">
-        <v>27</v>
+        <v>32</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
@@ -1263,7 +1263,7 @@
         <v>3490</v>
       </c>
       <c r="D3" t="s">
-        <v>28</v>
+        <v>33</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">
@@ -1271,7 +1271,7 @@
         <v>11</v>
       </c>
       <c r="B4" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="C4">
         <v>3500</v>
@@ -1299,7 +1299,7 @@
         <v>3525</v>
       </c>
       <c r="D6" t="s">
-        <v>29</v>
+        <v>34</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
Final touches on Figure 1 for Rmd
</commit_message>
<xml_diff>
--- a/R-Figs/AutoReadUSBRData/ReservoirElevationDefinitions.xlsx
+++ b/R-Figs/AutoReadUSBRData/ReservoirElevationDefinitions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://api.box.com/wopi/files/2558006682865/WOPIServiceId_TP_BOX_2/WOPIUserId_-/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="35" documentId="13_ncr:1_{93E988A9-6564-4F69-98E8-ABFBF40E39BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D577B65D-7E7C-41A5-A032-C630C2BCCC4D}"/>
+  <xr:revisionPtr revIDLastSave="41" documentId="13_ncr:1_{93E988A9-6564-4F69-98E8-ABFBF40E39BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D29A1D51-9FC6-4E2D-BE00-67012A1B5EF2}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{8459C475-5003-475B-AAB9-94E9EA45958F}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="35">
   <si>
     <t>Reservoir</t>
   </si>
@@ -136,10 +136,10 @@
     <t>No downstream delivery to;Lower Basin states and Mexico.</t>
   </si>
   <si>
-    <t>No hydropower generation or transmission; to 9 western U.S. states.;Infrastructure operates outside;design criteria.;Reduced downstream delivery to;Lower Basin states and Mexico.</t>
-  </si>
-  <si>
-    <t>Higher release temperatures.;Increased risk that invasive fish pass;though dam, spawn, spread, and;threaten native fish</t>
+    <t>No hydropower generation;or transmission to 9 states.;Infrastructure operates outside;design criteria.;Reduced downstream delivery.</t>
+  </si>
+  <si>
+    <t>Lower Equalization</t>
   </si>
 </sst>
 </file>
@@ -1217,7 +1217,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E38887C4-AA44-419C-B405-A9906CF058A2}">
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:D10"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="10.08984375" customWidth="1"/>
@@ -1298,19 +1298,16 @@
       <c r="C6">
         <v>3525</v>
       </c>
-      <c r="D6" t="s">
-        <v>34</v>
-      </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>11</v>
       </c>
       <c r="B7" t="s">
-        <v>14</v>
+        <v>34</v>
       </c>
       <c r="C7">
-        <v>3575</v>
+        <v>3550</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.35">
@@ -1318,10 +1315,10 @@
         <v>11</v>
       </c>
       <c r="B8" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C8">
-        <v>3600</v>
+        <v>3575</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.35">
@@ -1329,12 +1326,23 @@
         <v>11</v>
       </c>
       <c r="B9" t="s">
+        <v>15</v>
+      </c>
+      <c r="C9">
+        <v>3600</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>11</v>
+      </c>
+      <c r="B10" t="s">
         <v>13</v>
       </c>
-      <c r="C9">
+      <c r="C10">
         <v>3700</v>
       </c>
-      <c r="D9" t="s">
+      <c r="D10" t="s">
         <v>13</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Figure 2 Lake Mead working in R and Rmd
</commit_message>
<xml_diff>
--- a/R-Figs/AutoReadUSBRData/ReservoirElevationDefinitions.xlsx
+++ b/R-Figs/AutoReadUSBRData/ReservoirElevationDefinitions.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://api.box.com/wopi/files/2558006682865/WOPIServiceId_TP_BOX_2/WOPIUserId_-/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="41" documentId="13_ncr:1_{93E988A9-6564-4F69-98E8-ABFBF40E39BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D29A1D51-9FC6-4E2D-BE00-67012A1B5EF2}"/>
+  <xr:revisionPtr revIDLastSave="56" documentId="13_ncr:1_{93E988A9-6564-4F69-98E8-ABFBF40E39BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EA5FA72D-0C1F-440B-BD63-60CC2A055D0E}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{8459C475-5003-475B-AAB9-94E9EA45958F}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{8459C475-5003-475B-AAB9-94E9EA45958F}"/>
   </bookViews>
   <sheets>
     <sheet name="ReadMe" sheetId="2" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="36">
   <si>
     <t>Reservoir</t>
   </si>
@@ -118,21 +118,12 @@
     <t>Consequence</t>
   </si>
   <si>
-    <t>No downstream delivery to CA, AZ, and Mexico</t>
-  </si>
-  <si>
-    <t>No hydropower generation and delivery to;Los Angeles, Las Vegas, or Phoenix</t>
-  </si>
-  <si>
     <t>Minimum Drawdown Elevation (2026)</t>
   </si>
   <si>
     <t>Minimum Drawdown Elevations (2026)</t>
   </si>
   <si>
-    <t>Invasive fish stop moving upstream into Grand Canyon;Potect native fish</t>
-  </si>
-  <si>
     <t>No downstream delivery to;Lower Basin states and Mexico.</t>
   </si>
   <si>
@@ -140,6 +131,18 @@
   </si>
   <si>
     <t>Lower Equalization</t>
+  </si>
+  <si>
+    <t>Invasive fish stop moving;upstream into Grand Canyon.</t>
+  </si>
+  <si>
+    <t>No downstream delivery to;CA, AZ, and Mexico.</t>
+  </si>
+  <si>
+    <t>No hydropower generation or;transmission to Los Angeles, Las Vegas,;or Phoenix</t>
+  </si>
+  <si>
+    <t>Generate and transmit;29% of rated hydropower</t>
   </si>
 </sst>
 </file>
@@ -1043,7 +1046,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A8FD67FD-F240-49E2-BF91-7D417E153654}">
-  <dimension ref="A1:D13"/>
+  <dimension ref="A1:D14"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="16.90625" customWidth="1"/>
@@ -1074,7 +1077,7 @@
         <v>895</v>
       </c>
       <c r="D2" t="s">
-        <v>27</v>
+        <v>33</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
@@ -1088,7 +1091,7 @@
         <v>950</v>
       </c>
       <c r="D3" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">
@@ -1107,7 +1110,7 @@
         <v>1</v>
       </c>
       <c r="B5" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C5">
         <v>1000</v>
@@ -1139,11 +1142,11 @@
       <c r="A8" t="s">
         <v>1</v>
       </c>
-      <c r="B8" t="s">
-        <v>24</v>
-      </c>
       <c r="C8">
-        <v>1040</v>
+        <v>1035</v>
+      </c>
+      <c r="D8" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.35">
@@ -1151,10 +1154,10 @@
         <v>1</v>
       </c>
       <c r="B9" t="s">
-        <v>7</v>
+        <v>24</v>
       </c>
       <c r="C9">
-        <v>1050</v>
+        <v>1040</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.35">
@@ -1162,10 +1165,10 @@
         <v>1</v>
       </c>
       <c r="B10" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C10">
-        <v>1090</v>
+        <v>1050</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.35">
@@ -1173,13 +1176,10 @@
         <v>1</v>
       </c>
       <c r="B11" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C11">
-        <v>1135</v>
-      </c>
-      <c r="D11" t="s">
-        <v>31</v>
+        <v>1090</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.35">
@@ -1187,13 +1187,13 @@
         <v>1</v>
       </c>
       <c r="B12" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C12">
-        <v>1218</v>
+        <v>1135</v>
       </c>
       <c r="D12" t="s">
-        <v>10</v>
+        <v>32</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.35">
@@ -1201,12 +1201,23 @@
         <v>1</v>
       </c>
       <c r="B13" t="s">
+        <v>10</v>
+      </c>
+      <c r="C13">
+        <v>1218</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A14" t="s">
+        <v>1</v>
+      </c>
+      <c r="B14" t="s">
         <v>13</v>
       </c>
-      <c r="C13">
+      <c r="C14">
         <v>1220</v>
       </c>
-      <c r="D13" t="s">
+      <c r="D14" t="s">
         <v>13</v>
       </c>
     </row>
@@ -1249,7 +1260,7 @@
         <v>3370</v>
       </c>
       <c r="D2" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
@@ -1263,7 +1274,7 @@
         <v>3490</v>
       </c>
       <c r="D3" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">
@@ -1271,7 +1282,7 @@
         <v>11</v>
       </c>
       <c r="B4" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="C4">
         <v>3500</v>
@@ -1304,7 +1315,7 @@
         <v>11</v>
       </c>
       <c r="B7" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="C7">
         <v>3550</v>

</xml_diff>

<commit_message>
Figure 4 working in .R
</commit_message>
<xml_diff>
--- a/R-Figs/AutoReadUSBRData/ReservoirElevationDefinitions.xlsx
+++ b/R-Figs/AutoReadUSBRData/ReservoirElevationDefinitions.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://api.box.com/wopi/files/2558006682865/WOPIServiceId_TP_BOX_2/WOPIUserId_-/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="56" documentId="13_ncr:1_{93E988A9-6564-4F69-98E8-ABFBF40E39BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EA5FA72D-0C1F-440B-BD63-60CC2A055D0E}"/>
+  <xr:revisionPtr revIDLastSave="57" documentId="13_ncr:1_{93E988A9-6564-4F69-98E8-ABFBF40E39BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{79F16739-B939-47D2-8CFF-3E41A03FE1CF}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{8459C475-5003-475B-AAB9-94E9EA45958F}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{8459C475-5003-475B-AAB9-94E9EA45958F}"/>
   </bookViews>
   <sheets>
     <sheet name="ReadMe" sheetId="2" r:id="rId1"/>
@@ -118,9 +118,6 @@
     <t>Consequence</t>
   </si>
   <si>
-    <t>Minimum Drawdown Elevation (2026)</t>
-  </si>
-  <si>
     <t>Minimum Drawdown Elevations (2026)</t>
   </si>
   <si>
@@ -143,6 +140,9 @@
   </si>
   <si>
     <t>Generate and transmit;29% of rated hydropower</t>
+  </si>
+  <si>
+    <t>Minimum Drawdown;Elevation (2026)</t>
   </si>
 </sst>
 </file>
@@ -1077,7 +1077,7 @@
         <v>895</v>
       </c>
       <c r="D2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
@@ -1091,7 +1091,7 @@
         <v>950</v>
       </c>
       <c r="D3" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">
@@ -1110,7 +1110,7 @@
         <v>1</v>
       </c>
       <c r="B5" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C5">
         <v>1000</v>
@@ -1146,7 +1146,7 @@
         <v>1035</v>
       </c>
       <c r="D8" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.35">
@@ -1193,7 +1193,7 @@
         <v>1135</v>
       </c>
       <c r="D12" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.35">
@@ -1260,7 +1260,7 @@
         <v>3370</v>
       </c>
       <c r="D2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
@@ -1274,7 +1274,7 @@
         <v>3490</v>
       </c>
       <c r="D3" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">
@@ -1282,7 +1282,7 @@
         <v>11</v>
       </c>
       <c r="B4" t="s">
-        <v>27</v>
+        <v>35</v>
       </c>
       <c r="C4">
         <v>3500</v>
@@ -1315,7 +1315,7 @@
         <v>11</v>
       </c>
       <c r="B7" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C7">
         <v>3550</v>

</xml_diff>